<commit_message>
Update budget variance tracker workbook
</commit_message>
<xml_diff>
--- a/03_budget_variance_tracker/Program_Budget_Variance_Tracker.xlsx
+++ b/03_budget_variance_tracker/Program_Budget_Variance_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A46D4A57-22D4-4301-A5EB-A86E678E1FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481161D0-9DAA-48E5-B7EB-9C742EB5974C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="88">
   <si>
     <t>Program Budget &amp; Cost Variance Tracker</t>
   </si>
@@ -156,24 +156,6 @@
     <t>Total Bid ($K)</t>
   </si>
   <si>
-    <t>How to build this as an Excel Scenario (do this live in Excel):</t>
-  </si>
-  <si>
-    <t>1. Select cells B5:B7 (Bid A's inputs).</t>
-  </si>
-  <si>
-    <t>2. Data tab &gt; What-If Analysis &gt; Scenario Manager &gt; Add.</t>
-  </si>
-  <si>
-    <t>3. Name it 'Bid A', confirm the changing cells are B5:B7, click OK, enter the Bid A values, OK.</t>
-  </si>
-  <si>
-    <t>4. Repeat for Bid B (cells C5:C7) and Bid C (cells D5:D7).</t>
-  </si>
-  <si>
-    <t>5. Click 'Summary' in Scenario Manager to auto-generate a comparison report showing Total Bid under each scenario.</t>
-  </si>
-  <si>
     <t>Budget Cap Scenario</t>
   </si>
   <si>
@@ -196,24 +178,6 @@
   </si>
   <si>
     <t>Target: Total Bid should equal the Contingency Budget above</t>
-  </si>
-  <si>
-    <t>How to run Goal Seek (do this live in Excel):</t>
-  </si>
-  <si>
-    <t>1. Data tab &gt; What-If Analysis &gt; Goal Seek.</t>
-  </si>
-  <si>
-    <t>2. Set cell: B9 (Resulting Total Bid).</t>
-  </si>
-  <si>
-    <t>3. To value: type the number currently in B4 (Remaining Contingency Budget).</t>
-  </si>
-  <si>
-    <t>4. By changing cell: B8 (Labor Rate).</t>
-  </si>
-  <si>
-    <t>5. Click OK. Excel solves backward for the max labor rate I can afford without blowing the budget cap.</t>
   </si>
   <si>
     <t>Bibliography / Sources</t>
@@ -521,22 +485,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -565,6 +524,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -840,58 +803,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>97</v>
+      <c r="B4" s="5" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="150" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>98</v>
+      <c r="B6" s="5" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="135" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="s">
-        <v>99</v>
+      <c r="B8" s="23" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="6"/>
-      <c r="B14" s="7"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -910,223 +873,223 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="6">
         <v>1</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="9">
         <v>200</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="9">
         <v>235</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="10">
         <f t="shared" ref="D7:E11" si="0">B7*$B$4</f>
         <v>200</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="10">
         <f t="shared" si="0"/>
         <v>235</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="10">
         <f>E7-D7</f>
         <v>35</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="11">
         <f t="shared" ref="G7:G12" si="1">IF(D7=0,0,F7/D7)</f>
         <v>0.17499999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="9">
         <v>120</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="9">
         <v>140</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="10">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="10">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="10">
         <f>E8-D8</f>
         <v>20</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="11">
         <f t="shared" si="1"/>
         <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="9">
         <v>80</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="9">
         <v>75</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="10">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="10">
         <f t="shared" si="0"/>
         <v>75</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="10">
         <f>E9-D9</f>
         <v>-5</v>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="11">
         <f t="shared" si="1"/>
         <v>-6.25E-2</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="9">
         <v>60</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="9">
         <v>65</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="10">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="10">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="10">
         <f>E10-D10</f>
         <v>5</v>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="11">
         <f t="shared" si="1"/>
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="9">
         <v>40</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="9">
         <v>10</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="10">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="10">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="10">
         <f>E11-D11</f>
         <v>-30</v>
       </c>
-      <c r="G11" s="14">
+      <c r="G11" s="11">
         <f t="shared" si="1"/>
         <v>-0.75</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="13">
         <f>SUM(B7:B11)</f>
         <v>500</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="13">
         <f>SUM(C7:C11)</f>
         <v>525</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="13">
         <f>SUM(D7:D11)</f>
         <v>500</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="13">
         <f>SUM(E7:E11)</f>
         <v>525</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="13">
         <f>SUM(F7:F11)</f>
         <v>25</v>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="14">
         <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1139,7 +1102,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1147,170 +1110,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="9">
         <v>145</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="9">
         <v>160</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="9">
         <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="15">
         <v>4000</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="15">
         <v>3400</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="15">
         <v>4600</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="9">
         <v>210</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="9">
         <v>195</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="9">
         <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="15">
         <v>14</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="15">
         <v>11</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="15">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="17">
         <f>(B5*B6)/1000+B7</f>
         <v>790</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="17">
         <f>(C5*C6)/1000+C7</f>
         <v>739</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="17">
         <f>(D5*D6)/1000+D7</f>
         <v>823</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A16:F16"/>
+  <mergeCells count="1">
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1319,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1327,113 +1233,63 @@
     <col min="3" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:2" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="15">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="15">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="6">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="19" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="9">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="18">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="18">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="9">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="20">
+      <c r="B9" s="17">
         <f>(B8*B5)/1000+B6</f>
         <v>790</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>45</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1452,176 +1308,176 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="20">
+        <v>1</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="20">
+        <v>2</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="22" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="D6" s="22" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+      <c r="E6" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="10" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="20">
+        <v>3</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C7" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D7" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E7" s="22" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="23">
-        <v>1</v>
-      </c>
-      <c r="B5" s="24" t="s">
+    <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="20">
+        <v>4</v>
+      </c>
+      <c r="B8" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C8" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D8" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="25" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="20">
+        <v>5</v>
+      </c>
+      <c r="B9" s="21" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="23">
-        <v>2</v>
-      </c>
-      <c r="B6" s="24" t="s">
+      <c r="C9" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="D9" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="E9" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="25" t="s">
+    </row>
+    <row r="10" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="20">
+        <v>6</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="23">
-        <v>3</v>
-      </c>
-      <c r="B7" s="24" t="s">
+      <c r="C10" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="D10" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="E10" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E7" s="25" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="20">
+        <v>7</v>
+      </c>
+      <c r="B11" s="21" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="23">
-        <v>4</v>
-      </c>
-      <c r="B8" s="24" t="s">
+      <c r="C11" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="D11" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="D8" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="25" t="s">
+      <c r="E11" s="22" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="23">
-        <v>5</v>
-      </c>
-      <c r="B9" s="24" t="s">
+    <row r="12" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="20">
+        <v>8</v>
+      </c>
+      <c r="B12" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C12" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D12" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E12" s="22" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="23">
-        <v>6</v>
-      </c>
-      <c r="B10" s="24" t="s">
+    <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="C10" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="D10" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="E10" s="25" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="23">
-        <v>7</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="D11" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="23">
-        <v>8</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="E12" s="25" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>